<commit_message>
Capabilities workbook v2.1 — apply review (A-grade) changes
Per the review: (1) removed 'mission-driven organizations' everywhere -> 'communities,
public-sector organizations, and community-serving institutions' (workbook + deck);
(2) added a 'CLIENTS BUY / WE DELIVER' positioning block (funding/progress/capacity/
execution -> Institutional Stewardship = the business model); (3) added CAPACITY SUPPORT
as the 4th service line + 4th signature offering (interim/fractional/special-project/
admin/program coordination — Swanzey/Hubbardston/Sutton/Michigan LTC); (4) rebuilt the
Target Pipeline as a ranked DECISION TOOL — Authority / Relationship / Revenue Potential /
Probability / live Weighted Value (Revenue x Probability) / Next Action; sort to rank,
commit to top 5/month. Live formulas, zero errors.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000F4C3A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="000F4C3A"/>
       <sz val="12"/>
     </font>
@@ -68,7 +76,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +101,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3EAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -122,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,16 +156,28 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -520,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -549,7 +574,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>PublicLogic applies Institutional Stewardship to help communities and mission-driven organizations move important projects from planning to implementation.</t>
+          <t>PublicLogic applies Institutional Stewardship to help communities, public-sector organizations, and community-serving institutions move important projects from planning to implementation.</t>
         </is>
       </c>
     </row>
@@ -580,34 +605,46 @@
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>POSITIONING STATEMENT</t>
+          <t>CLIENTS BUY / WE DELIVER</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>PublicLogic helps communities and mission-driven organizations move important projects from planning to implementation. We do this through Institutional Stewardship — preserving, governing, transferring, and operationalizing the knowledge required for long-term success.</t>
+          <t>Clients buy funding, progress, capacity, and execution. PublicLogic delivers Institutional Stewardship. That is not a contradiction — it is the business model.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>INSTITUTIONAL STEWARDSHIP (definition)</t>
+          <t>POSITIONING STATEMENT</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The deliberate practice of preserving, governing, transferring, and operationalizing organizational knowledge so critical functions remain durable across turnover, changing priorities, and organizational change. An operating discipline, applied to every engagement regardless of project type.</t>
+          <t>PublicLogic helps communities, public-sector organizations, and community-serving institutions move important projects from planning to implementation. We do this through Institutional Stewardship — preserving, governing, transferring, and operationalizing the knowledge required for long-term success.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>INSTITUTIONAL STEWARDSHIP (definition)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>The deliberate practice of preserving, governing, transferring, and operationalizing organizational knowledge so critical functions remain durable across turnover, changing priorities, and organizational change. An operating discipline, applied to every engagement regardless of project type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>SUCCESS STANDARD</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>A successful engagement reduces future dependency. The organization becomes more capable; the process more durable; the knowledge more accessible.</t>
         </is>
@@ -624,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -756,6 +793,33 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Capacity Support</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Provide the institutional capacity to carry the work — directly.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Interim / fractional support · special-project support · administrative capacity · program coordination  (Swanzey · Hubbardston · Sutton · Michigan LTC)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Embedded Capacity Plan · Role / Coverage Map · Coordination Cadence · Continuity Handoff</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Hold the Chair so critical functions stay covered through turnover and transition.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -767,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -883,6 +947,26 @@
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Capacity Support Engagement</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Provide interim / fractional capacity to carry a function or special project.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Embedded Capacity Plan + Continuity Handoff</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1127,15 +1211,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1148,7 +1234,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Prioritize organizations that already have projects and budgets. Yellow = working pipeline fields.</t>
+          <t>A decision tool, not a list. Fill yellow cells; Weighted Value = Revenue x Probability. Sort by Weighted Value (descending) to rank.</t>
         </is>
       </c>
     </row>
@@ -1160,27 +1246,37 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Named Target</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Why / Need</t>
+          <t>Authority to Buy</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Relationship</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Revenue Potential ($)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Next Step</t>
+          <t>Probability</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Weighted Value ($)</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Next Action</t>
         </is>
       </c>
     </row>
@@ -1195,14 +1291,22 @@
           <t>CMRPC</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Municipal implementation support; active project pipelines</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Yes — active contracts &amp; pipelines</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Developing</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr"/>
+      <c r="F5" s="11" t="inlineStr"/>
+      <c r="G5" s="12">
+        <f>IF(AND(ISNUMBER(E5),ISNUMBER(F5)),E5*F5,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1215,14 +1319,22 @@
           <t>MRPC</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Delivery capacity; community engagement</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Yes — active pipelines</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Developing</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="12">
+        <f>IF(AND(ISNUMBER(E6),ISNUMBER(F6)),E6*F6,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1235,14 +1347,22 @@
           <t>MVPC</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Project delivery capacity</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Yes — project pipelines</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="12">
+        <f>IF(AND(ISNUMBER(E7),ISNUMBER(F7)),E7*F7,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1255,14 +1375,22 @@
           <t>Strafford RPC</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Municipal implementation support</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="12">
+        <f>IF(AND(ISNUMBER(E8),ISNUMBER(F8)),E8*F8,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1275,14 +1403,22 @@
           <t>Fuss &amp; O'Neill</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Public-process support; funding narratives; municipal coordination</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Yes — buys as sub/teaming</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr"/>
+      <c r="G9" s="12">
+        <f>IF(AND(ISNUMBER(E9),ISNUMBER(F9)),E9*F9,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1295,14 +1431,22 @@
           <t>Weston &amp; Sampson</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Municipal implementation capacity</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Yes — teaming</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="12">
+        <f>IF(AND(ISNUMBER(E10),ISNUMBER(F10)),E10*F10,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1315,14 +1459,22 @@
           <t>Tighe &amp; Bond</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Public process + funding narratives</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Yes — teaming</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="12">
+        <f>IF(AND(ISNUMBER(E11),ISNUMBER(F11)),E11*F11,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1335,14 +1487,22 @@
           <t>BETA</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Municipal coordination capacity</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Yes — teaming</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="12">
+        <f>IF(AND(ISNUMBER(E12),ISNUMBER(F12)),E12*F12,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1352,17 +1512,25 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Community Paradigm (and similar)</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Capacity + specialized expertise; subcontracting path</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+          <t>Community Paradigm (+ similar)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Yes — subcontract</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
+      <c r="G13" s="12">
+        <f>IF(AND(ISNUMBER(E13),ISNUMBER(F13)),E13*F13,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1372,17 +1540,25 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>(by relationship)</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Temporary capacity, strategic initiatives, capital planning, funding</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr"/>
-      <c r="F14" s="9" t="inlineStr"/>
+          <t>Direct (by relationship)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Yes — direct budget</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Warm — existing (Sutton/Shrewsbury/Phillipston)</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="12">
+        <f>IF(AND(ISNUMBER(E14),ISNUMBER(F14)),E14*F14,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1392,29 +1568,46 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>(warm relationships)</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Highest trust, shortest sales cycle</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>BD principle: don't convince organizations they have a hidden problem — help them solve a known one. Lead with capacity, funding, progress, execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+          <t>Warm relationships</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Strong — warmest, shortest cycle</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="12">
+        <f>IF(AND(ISNUMBER(E15),ISNUMBER(F15)),E15*F15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>How to use: enter Revenue Potential ($) and Probability (%) for each target; Weighted Value computes automatically; sort the table by Weighted Value descending to rank. Then commit to the top 5 for the month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>BD principle: don't convince organizations they have a hidden problem — help them solve a known one. Lead with capacity, funding, progress, execution. Warmest relationships first (shortest sales cycle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A18:F19"/>
+  <mergeCells count="2">
+    <mergeCell ref="A17:H18"/>
+    <mergeCell ref="A19:H20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1508,7 +1701,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Key insight: lead with the known problem, not a hidden one. The method (Institutional Stewardship) is how we deliver — outcomes are why they buy.</t>
         </is>
@@ -1543,38 +1736,38 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>PublicLogic is not in the business of producing reports.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>PublicLogic is not in the business of producing plans that sit on shelves.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>PublicLogic is in the business of helping organizations move important work forward — while ensuring the knowledge, systems, and structures required to sustain that work remain intact.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="inlineStr"/>
+      <c r="A7" s="17" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Internal strategic principle:</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>The market buys project delivery. PublicLogic delivers Institutional Stewardship. Both statements are true. Neither should be sacrificed for the other.</t>
         </is>

</xml_diff>

<commit_message>
Capabilities workbook v2.3 — apply A-grade review (pipeline focus, service differentiation, pricing)
1. PIPELINE FOCUS: added a 'Pursue' column (NOW/Qualify/Later) and illustrative
   Revenue/Probability so Weighted Value ranks the list — top 5 surface as CMRPC,
   warm municipalities, MRPC, existing network, Fuss & O'Neill. First-pass focus note
   + instruction to replace placeholders with real figures and commit to top 5.
2. SERVICE DIFFERENTIATION: added 'Implementation Support vs Capacity Support — which
   one?' clarifier — implementation = help your team execute (Shrewsbury); capacity =
   PublicLogic holds the role directly (Swanzey).
3. PRICING BANDS: Signature Offerings now show typical Scope/Duration/Fee
   (8-35K sprint · 5-28K funding · .5-15K/mo implementation · day-rate/-12K/mo
   capacity), fixed/non-contingent, with a note. Zero formula errors.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,7 +73,19 @@
       <sz val="9"/>
     </font>
     <font>
+      <color rgb="001A1D20"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F4C3A"/>
+    </font>
+    <font>
+      <color rgb="006B6660"/>
+      <sz val="10"/>
     </font>
     <font>
       <i val="1"/>
@@ -189,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -212,7 +224,16 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -221,13 +242,11 @@
     <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -236,10 +255,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -819,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -978,7 +997,25 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Implementation Support vs Capacity Support — which one?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Implementation Support = we help YOUR team execute — facilitation, accountability, coordination; the work stays theirs (e.g., Shrewsbury). Capacity Support = PublicLogic steps IN and holds the role or function directly — interim / fractional; we carry it until it transfers back (e.g., Swanzey). Same stewardship discipline; different level of who holds the Chair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:E12"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -989,16 +1026,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1038,17 +1075,17 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>Scope (fill)</t>
+          <t>Scope (typical)</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Duration (fill)</t>
+          <t>Duration (typical)</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Fee (fill)</t>
+          <t>Fee (typical)</t>
         </is>
       </c>
     </row>
@@ -1073,9 +1110,21 @@
           <t>CaseSpace + reusable Charter/Scope template</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr"/>
-      <c r="F5" s="12" t="inlineStr"/>
-      <c r="G5" s="12" t="inlineStr"/>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Map + charter + roadmap, one initiative</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>4–6 weeks</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>$18K–$35K (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1098,9 +1147,21 @@
           <t>Reusable funding scan + roadmap workbook</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr"/>
-      <c r="F6" s="12" t="inlineStr"/>
-      <c r="G6" s="12" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Funding scan + roadmap + readiness</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>3–5 weeks</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>$15K–$28K (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1123,9 +1184,21 @@
           <t>VAULT continuity record + accountability structure</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr"/>
-      <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="12" t="inlineStr"/>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Coordination + accountability through delivery</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>6–18 months</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>$6.5K–$15K / month</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1148,11 +1221,34 @@
           <t>Role/Coverage Map + Continuity Handoff</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr"/>
-      <c r="F8" s="12" t="inlineStr"/>
-      <c r="G8" s="12" t="inlineStr"/>
-    </row>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Interim role / special-project capacity</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Ongoing / fractional</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Day rate or $4K–$12K / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Typical ranges to anchor a sales conversation — confirm per engagement. All fees are fixed-fee or retainer and non-contingent. Where federal/grant funds pay, the fee rides as an allowable professional-service cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:G11"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1561,17 +1657,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1584,370 +1681,485 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>A decision tool, not a list. Fill yellow cells; Weighted Value = Revenue x Probability. Sort to rank.</t>
+          <t>Decision tool. Revenue/Probability are ILLUSTRATIVE placeholders to show ranking — replace with your figures. Weighted Value = Revenue x Probability; sort descending to rank.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
+          <t>Pursue</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Authority to Buy</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Relationship</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Revenue Potential ($)</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Weighted Value ($)</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Next Action</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>CMRPC</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Yes — active contracts &amp; pipelines</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr"/>
-      <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="15">
-        <f>IF(AND(ISNUMBER(E5),ISNUMBER(F5)),E5*F5,0)</f>
+      <c r="F5" s="16" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H5" s="18">
+        <f>IF(AND(ISNUMBER(F5),ISNUMBER(G5)),F5*G5,0)</f>
         <v/>
       </c>
+      <c r="I5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>MRPC</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Yes — active pipelines</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr"/>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="15">
-        <f>IF(AND(ISNUMBER(E6),ISNUMBER(F6)),E6*F6,0)</f>
+      <c r="F6" s="16" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H6" s="18">
+        <f>IF(AND(ISNUMBER(F6),ISNUMBER(G6)),F6*G6,0)</f>
         <v/>
       </c>
+      <c r="I6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Qualify</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>MVPC</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Yes — project pipelines</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
-      <c r="G7" s="15">
-        <f>IF(AND(ISNUMBER(E7),ISNUMBER(F7)),E7*F7,0)</f>
+      <c r="F7" s="16" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H7" s="18">
+        <f>IF(AND(ISNUMBER(F7),ISNUMBER(G7)),F7*G7,0)</f>
         <v/>
       </c>
+      <c r="I7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Strafford RPC</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr"/>
-      <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="15">
-        <f>IF(AND(ISNUMBER(E8),ISNUMBER(F8)),E8*F8,0)</f>
+      <c r="F8" s="16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H8" s="18">
+        <f>IF(AND(ISNUMBER(F8),ISNUMBER(G8)),F8*G8,0)</f>
         <v/>
       </c>
+      <c r="I8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Fuss &amp; O'Neill</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Yes — buys as sub/teaming</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr"/>
-      <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="15">
-        <f>IF(AND(ISNUMBER(E9),ISNUMBER(F9)),E9*F9,0)</f>
+      <c r="F9" s="16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H9" s="18">
+        <f>IF(AND(ISNUMBER(F9),ISNUMBER(G9)),F9*G9,0)</f>
         <v/>
       </c>
+      <c r="I9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Qualify</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Weston &amp; Sampson</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Yes — teaming</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="15">
-        <f>IF(AND(ISNUMBER(E10),ISNUMBER(F10)),E10*F10,0)</f>
+      <c r="F10" s="16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H10" s="18">
+        <f>IF(AND(ISNUMBER(F10),ISNUMBER(G10)),F10*G10,0)</f>
         <v/>
       </c>
+      <c r="I10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Tighe &amp; Bond</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Yes — teaming</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="15">
-        <f>IF(AND(ISNUMBER(E11),ISNUMBER(F11)),E11*F11,0)</f>
+      <c r="F11" s="16" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H11" s="18">
+        <f>IF(AND(ISNUMBER(F11),ISNUMBER(G11)),F11*G11,0)</f>
         <v/>
       </c>
+      <c r="I11" s="13" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>BETA</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Yes — teaming</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="15">
-        <f>IF(AND(ISNUMBER(E12),ISNUMBER(F12)),E12*F12,0)</f>
+      <c r="F12" s="16" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H12" s="18">
+        <f>IF(AND(ISNUMBER(F12),ISNUMBER(G12)),F12*G12,0)</f>
         <v/>
       </c>
+      <c r="I12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Qualify</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Municipal Consulting</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Community Paradigm (+ similar)</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Yes — subcontract</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
-      <c r="G13" s="15">
-        <f>IF(AND(ISNUMBER(E13),ISNUMBER(F13)),E13*F13,0)</f>
+      <c r="F13" s="16" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H13" s="18">
+        <f>IF(AND(ISNUMBER(F13),ISNUMBER(G13)),F13*G13,0)</f>
         <v/>
       </c>
+      <c r="I13" s="13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Municipalities</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Direct (by relationship)</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>Yes — direct budget</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>Warm — existing (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="15">
-        <f>IF(AND(ISNUMBER(E14),ISNUMBER(F14)),E14*F14,0)</f>
+      <c r="F14" s="16" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H14" s="18">
+        <f>IF(AND(ISNUMBER(F14),ISNUMBER(G14)),F14*G14,0)</f>
         <v/>
       </c>
+      <c r="I14" s="13" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Existing Network</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Warm relationships</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Varies</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Strong — warmest, shortest cycle</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
-      <c r="G15" s="15">
-        <f>IF(AND(ISNUMBER(E15),ISNUMBER(F15)),E15*F15,0)</f>
+      <c r="F15" s="16" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H15" s="18">
+        <f>IF(AND(ISNUMBER(F15),ISNUMBER(G15)),F15*G15,0)</f>
         <v/>
       </c>
+      <c r="I15" s="13" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>How to use: enter Revenue Potential ($) and Probability (%) for each target; Weighted Value computes automatically; sort the table by Weighted Value descending to rank. Then commit to the top 5 for the month.</t>
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>First-pass focus (June): pursue NOW = CMRPC · MRPC · one lead engineering firm (Fuss &amp; O'Neill) · the warm municipal &amp; existing-network relationships. Qualify the rest through the engagement flow; don't chase 'Later' yet. Replace the illustrative Revenue/Probability with real figures, then sort by Weighted Value and commit to the top 5.</t>
         </is>
       </c>
     </row>
     <row r="18"/>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>BD principle: don't convince organizations they have a hidden problem — help them solve a known one. Lead with capacity, funding, progress, execution. Warmest relationships first (shortest sales cycle).</t>
         </is>
@@ -1967,7 +2179,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
@@ -1977,15 +2189,16 @@
           <t>A known trigger: turnover, a stalled project, a funding deadline, a capacity gap.</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="19" t="n"/>
-      <c r="G23" s="19" t="n"/>
-      <c r="H23" s="20" t="n"/>
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="22" t="n"/>
+      <c r="F23" s="22" t="n"/>
+      <c r="G23" s="22" t="n"/>
+      <c r="H23" s="22" t="n"/>
+      <c r="I23" s="23" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>Fit</t>
         </is>
@@ -1995,15 +2208,16 @@
           <t>Confirm authority, budget, and that it is a known problem we solve.</t>
         </is>
       </c>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
-      <c r="G24" s="19" t="n"/>
-      <c r="H24" s="20" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="22" t="n"/>
+      <c r="G24" s="22" t="n"/>
+      <c r="H24" s="22" t="n"/>
+      <c r="I24" s="23" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>Map</t>
         </is>
@@ -2013,15 +2227,16 @@
           <t>A paid scoping engagement — diagnosis + roadmap (the entry move).</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="19" t="n"/>
-      <c r="E25" s="19" t="n"/>
-      <c r="F25" s="19" t="n"/>
-      <c r="G25" s="19" t="n"/>
-      <c r="H25" s="20" t="n"/>
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="22" t="n"/>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="23" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
@@ -2031,15 +2246,16 @@
           <t>Deliver the project, funding, implementation, or capacity work.</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
-      <c r="G26" s="19" t="n"/>
-      <c r="H26" s="20" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="22" t="n"/>
+      <c r="F26" s="22" t="n"/>
+      <c r="G26" s="22" t="n"/>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="23" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Sustain</t>
         </is>
@@ -2049,15 +2265,16 @@
           <t>Transfer ownership; optional capacity / retainer so it runs without us.</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="19" t="n"/>
-      <c r="G27" s="19" t="n"/>
-      <c r="H27" s="20" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="22" t="n"/>
+      <c r="G27" s="22" t="n"/>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="23" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>Prove</t>
         </is>
@@ -2067,23 +2284,24 @@
           <t>Capture the evidence (Proof tab) — which becomes the next Signal.</t>
         </is>
       </c>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="19" t="n"/>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="20" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="22" t="n"/>
+      <c r="G28" s="22" t="n"/>
+      <c r="H28" s="22" t="n"/>
+      <c r="I28" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A17:H18"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="A19:H20"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="B28:H28"/>
-    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="A19:I20"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="A17:I18"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B26:I26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2177,7 +2395,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Key insight: lead with the known problem, not a hidden one. The method (Institutional Stewardship) is how we deliver — outcomes are why they buy.</t>
         </is>
@@ -2212,38 +2430,38 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>PublicLogic is not in the business of producing reports.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>PublicLogic is not in the business of producing plans that sit on shelves.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>PublicLogic is in the business of helping organizations move important work forward — while ensuring the knowledge, systems, and structures required to sustain that work remain intact.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="23" t="inlineStr"/>
+      <c r="A7" s="26" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Internal strategic principle:</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>The market buys project delivery. PublicLogic delivers Institutional Stewardship. Both statements are true. Neither should be sacrificed for the other.</t>
         </is>

</xml_diff>

<commit_message>
Add one-pager + 'Start Here' tab — make it swallowable
Answer to 'too much to swallow': lead with one page, keep the depth behind it.
- PublicLogic - One Pager.pptx: single slide — North Star, the bridge, what we do
  (4 services), why different, 'we prove it', and How to Start (Signal->...->Prove,
  begin with a paid Map). 30-second read.
- Capabilities Workbook: added a 'Start Here' summary as the FIRST tab so it opens
  simple; the 9 detailed tabs follow only if wanted.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -7,15 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positioning" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Catalog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signature Offerings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Model" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfer Assets" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proof" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline &amp; Flow" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons Learned" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Promise" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positioning" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Service Catalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signature Offerings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Model" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfer Assets" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proof" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline &amp; Flow" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons Learned" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Promise" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,6 +98,10 @@
       <sz val="13"/>
     </font>
     <font/>
+    <font>
+      <color rgb="001A1D20"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -201,13 +206,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -220,7 +229,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -626,6 +634,184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PUBLICLOGIC — Start Here</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The whole workbook on one page. Depth is in the tabs that follow — only if you want it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>North Star</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Every system should make it easier for the next person to do the right thing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>The bridge</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Implementation is the service. Institutional Stewardship is the method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Why different</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Most systems manage work. PublicLogic helps steward what has to survive the work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>What we do</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Project Development · Funding Strategy · Implementation Support · Capacity Support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>We prove it</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Continuity · record · readiness · adoption · outcome (see Proof).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>How to start</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Signal → Fit → Map → Build → Sustain → Prove. Begin with a paid Map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Where to look</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Positioning · Service Catalog · Signature Offerings (pricing) · Proof · Pipeline &amp; Flow.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>The PublicLogic Promise</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>PublicLogic is not in the business of producing reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>PublicLogic is not in the business of producing plans that sit on shelves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>PublicLogic is in the business of helping organizations move important work forward — while ensuring the knowledge, systems, and structures required to sustain that work remain intact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="27" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Internal strategic principle:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>The market buys project delivery. PublicLogic delivers Institutional Stewardship. Both statements are true. Neither should be sacrificed for the other.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -641,7 +827,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Institutional Stewardship through Project Delivery  ·  v2.0  ·  June 2026</t>
         </is>
@@ -653,7 +839,7 @@
           <t>NORTH STAR</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Every system should make it easier for the next person to do the right thing.</t>
         </is>
@@ -665,7 +851,7 @@
           <t>WHY WE'RE DIFFERENT</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Most systems manage work. PublicLogic helps steward what has to survive the work.</t>
         </is>
@@ -677,7 +863,7 @@
           <t>WHAT WE ARE</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>PublicLogic applies Institutional Stewardship to help communities, public-sector organizations, and community-serving institutions move important projects from planning to implementation.</t>
         </is>
@@ -689,7 +875,7 @@
           <t>THE DISTINCTION</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Implementation is the service. Institutional Stewardship is the method. The market buys project delivery; PublicLogic delivers Institutional Stewardship. Both are true; neither is sacrificed for the other.</t>
         </is>
@@ -701,7 +887,7 @@
           <t>CLIENTS BUY / WE DELIVER</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Clients buy funding, progress, capacity, and execution. PublicLogic delivers Institutional Stewardship. That is not a contradiction — it is the business model.</t>
         </is>
@@ -713,7 +899,7 @@
           <t>WHAT WE ARE NOT</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Not a grant-writing firm. Not an AI consulting firm. Not a traditional planning firm. We don't produce reports or plans that sit on shelves.</t>
         </is>
@@ -725,7 +911,7 @@
           <t>POSITIONING STATEMENT</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>PublicLogic helps communities, public-sector organizations, and community-serving institutions move important projects from planning to implementation. We do this through Institutional Stewardship — preserving, governing, transferring, and operationalizing the knowledge required for long-term success.</t>
         </is>
@@ -737,7 +923,7 @@
           <t>INSTITUTIONAL STEWARDSHIP (definition)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>The deliberate practice of preserving, governing, transferring, and operationalizing organizational knowledge so critical functions remain durable across turnover, changing priorities, and organizational change.</t>
         </is>
@@ -749,7 +935,7 @@
           <t>IN PLAIN TERMS</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Stewardship — caring for what must outlast any one person.   Continuity — the work keeps running through turnover.   Institutional memory — the organization remembers how and why.   Transfer — every engagement leaves reusable capability.   Why plans fail — capacity stops keeping pace with complexity.</t>
         </is>
@@ -761,67 +947,67 @@
           <t>SUCCESS STANDARD</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>A successful engagement reduces future dependency. The organization becomes more capable; the process more durable; the knowledge more accessible.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>HOW WE WORK</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Map   →   Embed   →   Encode   →   Sustain</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Map</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Surface how the work actually happens — roles, knowledge, dependencies, risks.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Embed</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Put the right structure into the live workflow, alongside the people who do the work.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Encode</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Capture the knowledge and rules so they outlast any individual.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Sustain</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Monitor adoption and transfer ownership so it runs without us.</t>
         </is>
@@ -832,7 +1018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -849,163 +1035,163 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Core Service Lines</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Three services, one discipline. Stewardship objective shown per line.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Common Engagements</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Deliverables</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Stewardship Objective</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Project Development</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Transform ideas, priorities, and challenges into actionable projects.</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Strategic initiatives · capital projects · community development · housing · infrastructure · program development</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Project Charter · Scope Definition · Stakeholder Map · Readiness Assessment · Action Roadmap</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Create clarity before resources are committed.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Funding Strategy</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Identify, organize, and pursue sustainable funding opportunities.</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Grant development · capital planning · funding roadmaps · partnership development · revenue strategy</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Funding Scan · Funding Roadmap · Application Support · Capital Strategy · Partner Coordination</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Align funding with long-term organizational capacity.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Implementation Support</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Move projects from planning into execution.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Strategic-plan implementation · capital project coordination · program launch · community engagement · readiness</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Implementation Framework · Accountability Structure · Progress Tracking · Facilitation · Stakeholder Coordination</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Ensure important work survives beyond its initial champions.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Capacity Support</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Provide the institutional capacity to carry the work — directly.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Interim / fractional support · special-project support · administrative capacity · program coordination  (Swanzey · Hubbardston · Sutton · Michigan LTC)</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Embedded Capacity Plan · Role / Coverage Map · Coordination Cadence · Continuity Handoff</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Hold the Chair so critical functions stay covered through turnover and transition.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Implementation Support vs Capacity Support — which one?</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Implementation Support = we help YOUR team execute — facilitation, accountability, coordination; the work stays theirs (e.g., Shrewsbury). Capacity Support = PublicLogic steps IN and holds the role or function directly — interim / fractional; we carry it until it transfers back (e.g., Swanzey). Same stewardship discipline; different level of who holds the Chair.</t>
         </is>
@@ -1020,7 +1206,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1039,206 +1225,206 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Signature Offerings</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Three ways to start. Yellow = fill in scope, duration, and fee per engagement.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Offering</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Transfer Asset Created</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Scope (typical)</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Duration (typical)</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>Fee (typical)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Project Development Sprint</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Move an idea into an actionable project.</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Project Development Roadmap</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>CaseSpace + reusable Charter/Scope template</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Map + charter + roadmap, one initiative</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>4–6 weeks</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>$18K–$35K (fixed)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Funding Strategy Sprint</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Identify realistic funding pathways and readiness requirements.</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Funding Roadmap</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Reusable funding scan + roadmap workbook</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Funding scan + roadmap + readiness</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>3–5 weeks</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>$15K–$28K (fixed)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Implementation Support Partnership</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Provide coordination and stewardship capacity through implementation.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Implementation Framework + Accountability Structure</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>VAULT continuity record + accountability structure</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Coordination + accountability through delivery</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>6–18 months</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>$6.5K–$15K / month</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Capacity Support Engagement</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Provide interim / fractional capacity to carry a function or special project.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Embedded Capacity Plan + Continuity Handoff</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Role/Coverage Map + Continuity Handoff</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Interim role / special-project capacity</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Ongoing / fractional</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Day rate or $4K–$12K / month</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Typical ranges to anchor a sales conversation — confirm per engagement. All fees are fixed-fee or retainer and non-contingent. Where federal/grant funds pay, the fee rides as an allowable professional-service cost.</t>
         </is>
@@ -1253,7 +1439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1268,78 +1454,78 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>The Nathan + Allie Model</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Institutional systems and human systems are interdependent — projects fail when either is ignored.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr"/>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Nathan — Institutional Systems</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Allie — Human Systems</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Expertise</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Municipal administration · finance · capital planning · procurement · grants · economic development · governance · project delivery</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Organizational readiness · stakeholder engagement · leadership development · program design · evaluation · behavioral systems · change management</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Experience</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Town Administrator · City Councilor · Town Clerk · Consultant</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Clinical leadership · organizational consulting · program development · workforce systems</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>The pairing</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Most firms understand systems OR people.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>PublicLogic is designed to understand both.</t>
         </is>
@@ -1350,7 +1536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1365,116 +1551,116 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Transfer Assets</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>A core principle of stewardship: every engagement creates reusable organizational assets.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Asset</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Leaves the client with</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>LogicCommons</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Shared frameworks, templates, and operational resources.</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Reusable standards</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Workbooks</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Structured implementation and planning guides.</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Repeatable process</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>CaseSpaces</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Project-specific operating environments.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>A governed record</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>PuddleJumper</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Process architecture and workflow infrastructure.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Operating continuity</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>VAULT</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Knowledge preservation and continuity framework.</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Durability across turnover</t>
         </is>
@@ -1485,7 +1671,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1501,146 +1687,146 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Proof — Evidence of Stewardship</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Stewardship is provable, not just stated. Five kinds of proof, each tied to a real engagement.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Proof</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>What it demonstrates to a buyer</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>How we show it</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Continuity proof</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>A function survives when the person who ran it leaves.</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Successor test + VAULT modules mapped to authority and stop-rules.</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Sutton TIF — the 30-day successor test the town would otherwise fail.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Record proof</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Every claim, number, and decision traces to a source.</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>CaseSpace + Source Register: source file → workbook row → output.</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Michigan LTC corridor record — line-for-line traceability.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Readiness proof</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>The organization can absorb and sustain the change.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Readiness Assessment + the Map deliverable before any build.</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Pre-build assessment that sequences what the org can actually carry.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Adoption proof</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Staff actually use the system — not just receive it.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>CFIR-structured adoption monitoring through implementation.</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Shrewsbury — human-systems support so the build is used, not shelved.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Outcome proof</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>The work moved forward and got funded.</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Funded applications + delivered projects, documented.</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Shrewsbury fiber, Sutton — funding secured and projects implemented.</t>
         </is>
@@ -1651,7 +1837,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1672,486 +1858,486 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Target Pipeline &amp; Engagement Flow</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Decision tool. Revenue/Probability are ILLUSTRATIVE placeholders to show ranking — replace with your figures. Weighted Value = Revenue x Probability; sort descending to rank.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pursue</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Authority to Buy</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Relationship</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Revenue Potential ($)</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>Weighted Value ($)</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="I4" s="12" t="inlineStr">
         <is>
           <t>Next Action</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>CMRPC</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Yes — active contracts &amp; pipelines</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <v>60000</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="18" t="n">
         <v>0.45</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="19">
         <f>IF(AND(ISNUMBER(F5),ISNUMBER(G5)),F5*G5,0)</f>
         <v/>
       </c>
-      <c r="I5" s="13" t="inlineStr"/>
+      <c r="I5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>MRPC</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Yes — active pipelines</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <v>50000</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="18" t="n">
         <v>0.4</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="19">
         <f>IF(AND(ISNUMBER(F6),ISNUMBER(G6)),F6*G6,0)</f>
         <v/>
       </c>
-      <c r="I6" s="13" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>MVPC</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Yes — project pipelines</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="17" t="n">
         <v>50000</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="19">
         <f>IF(AND(ISNUMBER(F7),ISNUMBER(G7)),F7*G7,0)</f>
         <v/>
       </c>
-      <c r="I7" s="13" t="inlineStr"/>
+      <c r="I7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Later</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Regional Planning Agencies</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Strafford RPC</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <v>40000</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="18" t="n">
         <v>0.15</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="19">
         <f>IF(AND(ISNUMBER(F8),ISNUMBER(G8)),F8*G8,0)</f>
         <v/>
       </c>
-      <c r="I8" s="13" t="inlineStr"/>
+      <c r="I8" s="14" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Fuss &amp; O'Neill</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Yes — buys as sub/teaming</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="17" t="n">
         <v>40000</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="19">
         <f>IF(AND(ISNUMBER(F9),ISNUMBER(G9)),F9*G9,0)</f>
         <v/>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
+      <c r="I9" s="14" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Weston &amp; Sampson</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Yes — teaming</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <v>40000</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="19">
         <f>IF(AND(ISNUMBER(F10),ISNUMBER(G10)),F10*G10,0)</f>
         <v/>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="14" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Later</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Tighe &amp; Bond</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Yes — teaming</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="17" t="n">
         <v>35000</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="18" t="n">
         <v>0.15</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="19">
         <f>IF(AND(ISNUMBER(F11),ISNUMBER(G11)),F11*G11,0)</f>
         <v/>
       </c>
-      <c r="I11" s="13" t="inlineStr"/>
+      <c r="I11" s="14" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Later</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Engineering Firms</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>BETA</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Yes — teaming</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="17" t="n">
         <v>35000</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <v>0.15</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="19">
         <f>IF(AND(ISNUMBER(F12),ISNUMBER(G12)),F12*G12,0)</f>
         <v/>
       </c>
-      <c r="I12" s="13" t="inlineStr"/>
+      <c r="I12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Municipal Consulting</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Community Paradigm (+ similar)</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Yes — subcontract</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="17" t="n">
         <v>30000</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="19">
         <f>IF(AND(ISNUMBER(F13),ISNUMBER(G13)),F13*G13,0)</f>
         <v/>
       </c>
-      <c r="I13" s="13" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Municipalities</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Direct (by relationship)</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Yes — direct budget</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Warm — existing (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="17" t="n">
         <v>35000</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G14" s="18" t="n">
         <v>0.6</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H14" s="19">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(G14)),F14*G14,0)</f>
         <v/>
       </c>
-      <c r="I14" s="13" t="inlineStr"/>
+      <c r="I14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Existing Network</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Warm relationships</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Varies</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Strong — warmest, shortest cycle</t>
         </is>
       </c>
-      <c r="F15" s="16" t="n">
+      <c r="F15" s="17" t="n">
         <v>25000</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="18" t="n">
         <v>0.65</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="19">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(G15)),F15*G15,0)</f>
         <v/>
       </c>
-      <c r="I15" s="13" t="inlineStr"/>
+      <c r="I15" s="14" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>First-pass focus (June): pursue NOW = CMRPC · MRPC · one lead engineering firm (Fuss &amp; O'Neill) · the warm municipal &amp; existing-network relationships. Qualify the rest through the engagement flow; don't chase 'Later' yet. Replace the illustrative Revenue/Probability with real figures, then sort by Weighted Value and commit to the top 5.</t>
         </is>
@@ -2159,7 +2345,7 @@
     </row>
     <row r="18"/>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>BD principle: don't convince organizations they have a hidden problem — help them solve a known one. Lead with capacity, funding, progress, execution. Warmest relationships first (shortest sales cycle).</t>
         </is>
@@ -2167,130 +2353,130 @@
     </row>
     <row r="20"/>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>ENGAGEMENT FLOW</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Signal → Fit → Map → Build → Sustain → Prove</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>A known trigger: turnover, a stalled project, a funding deadline, a capacity gap.</t>
         </is>
       </c>
-      <c r="C23" s="22" t="n"/>
-      <c r="D23" s="22" t="n"/>
-      <c r="E23" s="22" t="n"/>
-      <c r="F23" s="22" t="n"/>
-      <c r="G23" s="22" t="n"/>
-      <c r="H23" s="22" t="n"/>
-      <c r="I23" s="23" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="23" t="n"/>
+      <c r="I23" s="24" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>Fit</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Confirm authority, budget, and that it is a known problem we solve.</t>
         </is>
       </c>
-      <c r="C24" s="22" t="n"/>
-      <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
-      <c r="F24" s="22" t="n"/>
-      <c r="G24" s="22" t="n"/>
-      <c r="H24" s="22" t="n"/>
-      <c r="I24" s="23" t="n"/>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
+      <c r="F24" s="23" t="n"/>
+      <c r="G24" s="23" t="n"/>
+      <c r="H24" s="23" t="n"/>
+      <c r="I24" s="24" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>Map</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>A paid scoping engagement — diagnosis + roadmap (the entry move).</t>
         </is>
       </c>
-      <c r="C25" s="22" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
-      <c r="F25" s="22" t="n"/>
-      <c r="G25" s="22" t="n"/>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="23" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="23" t="n"/>
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="23" t="n"/>
+      <c r="I25" s="24" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Deliver the project, funding, implementation, or capacity work.</t>
         </is>
       </c>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="22" t="n"/>
-      <c r="E26" s="22" t="n"/>
-      <c r="F26" s="22" t="n"/>
-      <c r="G26" s="22" t="n"/>
-      <c r="H26" s="22" t="n"/>
-      <c r="I26" s="23" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+      <c r="F26" s="23" t="n"/>
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="23" t="n"/>
+      <c r="I26" s="24" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>Sustain</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Transfer ownership; optional capacity / retainer so it runs without us.</t>
         </is>
       </c>
-      <c r="C27" s="22" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="22" t="n"/>
-      <c r="F27" s="22" t="n"/>
-      <c r="G27" s="22" t="n"/>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="23" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="23" t="n"/>
+      <c r="E27" s="23" t="n"/>
+      <c r="F27" s="23" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="23" t="n"/>
+      <c r="I27" s="24" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>Prove</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Capture the evidence (Proof tab) — which becomes the next Signal.</t>
         </is>
       </c>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
-      <c r="F28" s="22" t="n"/>
-      <c r="G28" s="22" t="n"/>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="F28" s="23" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="23" t="n"/>
+      <c r="I28" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2307,7 +2493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2321,81 +2507,81 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Lessons Learned · AI for Impact</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>People buy outcomes. The methodology matters, but outcomes drive the purchasing decision.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>What we thought they wanted</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>What they actually want</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Innovation</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Funding</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Readiness</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Transformation</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Execution</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Key insight: lead with the known problem, not a hidden one. The method (Institutional Stewardship) is how we deliver — outcomes are why they buy.</t>
         </is>
@@ -2408,66 +2594,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>The PublicLogic Promise</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>PublicLogic is not in the business of producing reports.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
-        <is>
-          <t>PublicLogic is not in the business of producing plans that sit on shelves.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>PublicLogic is in the business of helping organizations move important work forward — while ensuring the knowledge, systems, and structures required to sustain that work remain intact.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="26" t="inlineStr"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Internal strategic principle:</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>The market buys project delivery. PublicLogic delivers Institutional Stewardship. Both statements are true. Neither should be sacrificed for the other.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Permit & Bridge public/sponsor layers + Stewardship Map scope sheet
Permit & Bridge tab now carries the two-sided framing (Public Help Layer /
Project Sponsor Layer), the Public Output Layer (a guided public framework,
not AI consulting), and the Tier 0-5 Offer Ladder:
  0 Public Permit Helper (free/low) · 1 Permit Path Scan ($250-750) ·
  2 Stewardship Map ($2.5-7.5k) · 3 Permit & Bridge Sprint ($7.5-15k) ·
  4 White-Glove Implementation ($3.5-8.5k/mo) · 5 Funding/Grant Build ($5-25k).
Offer Stack notes the new public-facing entry rungs.

Adds build_stewardship_map_scope.py -> a sellable one-page Scope & Fee Sheet
(.docx) for the Stewardship Map: what it is, what we look at, what you get,
fixed non-contingent fee, why start here. Ready to send a Tier-1 prospect.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -200,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -232,6 +232,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -933,7 +936,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -943,24 +946,24 @@
           <t>CMRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <v>60000</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="21" t="n">
         <v>0.45</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="22">
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(E11)),D11*E11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -970,24 +973,24 @@
           <t>MRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="20" t="n">
         <v>50000</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="22">
         <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),D12*E12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -997,24 +1000,24 @@
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="20" t="n">
         <v>35000</v>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="21" t="n">
         <v>0.6</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="22">
         <f>IF(AND(ISNUMBER(D13),ISNUMBER(E13)),D13*E13,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1024,24 +1027,24 @@
           <t>Existing network</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>Strongest</t>
         </is>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="20" t="n">
         <v>25000</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="21" t="n">
         <v>0.65</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="22">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(E14)),D14*E14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1051,24 +1054,24 @@
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="20" t="n">
         <v>40000</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="21" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="22">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(E15)),D15*E15,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1078,24 +1081,24 @@
           <t>MVPC / other RPCs</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="20" t="n">
         <v>50000</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="22">
         <f>IF(AND(ISNUMBER(D16),ISNUMBER(E16)),D16*E16,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1105,18 +1108,18 @@
           <t>Community Paradigm (municipal consulting)</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="20" t="n">
         <v>30000</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="22">
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(E17)),D17*E17,0)</f>
         <v/>
       </c>
@@ -1144,10 +1147,10 @@
           <t>A known trigger: turnover, a stalled project, a funding deadline, a capacity gap.</t>
         </is>
       </c>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="23" t="n"/>
+      <c r="C20" s="23" t="n"/>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" s="24" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
@@ -1160,10 +1163,10 @@
           <t>Confirm authority, budget, and that it's a known problem we solve.</t>
         </is>
       </c>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="22" t="n"/>
-      <c r="F21" s="23" t="n"/>
+      <c r="C21" s="23" t="n"/>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="24" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
@@ -1176,10 +1179,10 @@
           <t>A paid Stewardship Map — the entry move.</t>
         </is>
       </c>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
-      <c r="F22" s="23" t="n"/>
+      <c r="C22" s="23" t="n"/>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="24" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
@@ -1192,10 +1195,10 @@
           <t>Deliver the project, funding, permit, implementation, or capacity work.</t>
         </is>
       </c>
-      <c r="C23" s="22" t="n"/>
-      <c r="D23" s="22" t="n"/>
-      <c r="E23" s="22" t="n"/>
-      <c r="F23" s="23" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="24" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -1208,10 +1211,10 @@
           <t>Transfer ownership; optional Implementation or Capacity Support.</t>
         </is>
       </c>
-      <c r="C24" s="22" t="n"/>
-      <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
-      <c r="F24" s="23" t="n"/>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
+      <c r="F24" s="24" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
@@ -1224,10 +1227,10 @@
           <t>Capture the evidence — which becomes the next Signal.</t>
         </is>
       </c>
-      <c r="C25" s="22" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
-      <c r="F25" s="23" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1780,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2001,8 +2004,17 @@
       </c>
     </row>
     <row r="12"/>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Entry below the Map: the Permit &amp; Bridge tab adds a public-facing ladder — Tier 0 Public Permit Helper (free / very low cost) and Tier 1 Permit Path Scan ($250–$750) — that builds trust and feeds these paid offers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A13:E14"/>
     <mergeCell ref="A11:E12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2015,11 +2027,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="104" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2032,11 +2045,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>This may be the most important thing we do.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="46" customHeight="1">
+          <t>This may be the most important thing we do.  Best line: Permit &amp; Bridge helps the public understand the path and helps project sponsors move through it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>What it is</t>
@@ -2044,11 +2057,11 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>PublicLogic helps project sponsors move through public systems.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="46" customHeight="1">
+          <t>PublicLogic helps project sponsors move through public systems — and helps the public understand the path before they get there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>That includes</t>
@@ -2060,7 +2073,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Why it exists</t>
@@ -2072,7 +2085,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>What we become</t>
@@ -2084,7 +2097,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Why it matters to us</t>
@@ -2096,7 +2109,278 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TWO SIDES OF THE SAME BRIDGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Audience</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Public Help Layer</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Residents · small owners · nonprofits</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>“Can I do X in my backyard / property / building?”  Cheap, simple, framework-guided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Project Sponsor Layer</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Developers · towns · nonprofits · businesses</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>White-glove permit path · stewardship map · grant / funding strategy · implementation support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>PERMIT &amp; BRIDGE: PUBLIC OUTPUT LAYER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>The free/cheap tier is NOT AI consulting. It is a guided public framework that helps people understand the path. PublicLogic can support a simple public-facing assistance layer for common questions:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>•  “Can I put this in my backyard?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>•  “Do I need a permit?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>•  “Who do I ask first?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>•  “What board or office handles this?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>•  “What documents will I likely need?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>•  “Is this a zoning, building, health, conservation, or licensing issue?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>This layer should be low-cost or free — its purpose is access, trust, and triage. It does NOT replace the municipality, inspector, planner, or permitting authority. It helps people ask better questions, gather the right information, and avoid wasting time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>THE OFFER LADDER  —  free tier creates trust; paid tiers handle complexity</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Public Permit Helper / “Can I Do This?”</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Free or very low cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Permit Path Scan</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>$250 – $750</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Stewardship Map</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>$2,500 – $7,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Permit &amp; Bridge Sprint</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>$7,500 – $15,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>White-Glove Implementation</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>$3,500 – $8,500 / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Funding / Grant Build</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>$5,000 – $25,000 (scope-dependent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Permit &amp; Bridge helps the public understand the path and helps project sponsors move through it.  That's the full product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
   </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A16:C17"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A37:C38"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2447,14 +2731,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>PublicLogic should be stronger after every engagement.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>The client should be less dependent after every engagement.</t>
         </is>

</xml_diff>

<commit_message>
Add LogicCommons public-access layer + Permit Path Scan scope sheet
Permit & Bridge tab now frames the full free-to-white-glove ladder around
LogicCommons as the public access layer (free templates/checklists/frameworks),
with the four-layer table (Free public tools / Cheap triage / Paid diagnostic /
White-glove help) and the core line: "LogicCommons helps people start.
PublicLogic helps them carry it through." Start Here carries the same line.

Adds build_permit_path_scan_scope.py -> a sellable one-page Scope & Fee Sheet
(.docx) for the Tier-1 Permit Path Scan ($250-750): where it sits, what it
answers, what you get, flat fee that credits toward the Map, and what it is NOT.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -200,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -232,6 +232,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -615,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -675,118 +678,130 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>1 · Why we exist</t>
+          <t>The ladder</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Good work keeps failing when knowledge, ownership, or continuity disappears. We've watched it happen, and we built the practices to stop it.</t>
+          <t>LogicCommons helps people start. PublicLogic helps them carry it through.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2 · The problem</t>
+          <t>1 · Why we exist</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Capacity stops keeping pace with complexity. The 'Chair' — the place where a function lives — ends up depending on one person.</t>
+          <t>Good work keeps failing when knowledge, ownership, or continuity disappears. We've watched it happen, and we built the practices to stop it.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>3 · What clients buy</t>
+          <t>2 · The problem</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Projects moved forward. Funding found and won. A role or function covered.</t>
+          <t>Capacity stops keeping pace with complexity. The 'Chair' — the place where a function lives — ends up depending on one person.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>4 · What we deliver</t>
+          <t>3 · What clients buy</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>The same — plus the stewardship that makes it survive turnover.</t>
+          <t>Projects moved forward. Funding found and won. A role or function covered.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>5 · What makes us different</t>
+          <t>4 · What we deliver</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Most systems manage work. PublicLogic helps steward what has to survive the work.</t>
+          <t>The same — plus the stewardship that makes it survive turnover.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>6 · What we sell</t>
+          <t>5 · What makes us different</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Stewardship Map (the safe first step) → Sprints (Project · Funding · Permit &amp; Bridge) → Implementation &amp; Capacity Support.</t>
+          <t>Most systems manage work. PublicLogic helps steward what has to survive the work.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>7 · Who first</t>
+          <t>6 · What we sell</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Our existing municipal network, regional planning agencies, engineering firms, municipal consulting firms.</t>
+          <t>Stewardship Map (the safe first step) → Sprints (Project · Funding · Permit &amp; Bridge) → Implementation &amp; Capacity Support.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>8 · How it compounds</t>
+          <t>7 · Who first</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Every engagement leaves reusable knowledge, templates, and proof. We get stronger; clients get less dependent.</t>
+          <t>Our existing municipal network, regional planning agencies, engineering firms, municipal consulting firms.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>9 · Nathan + Allie</t>
+          <t>8 · How it compounds</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Institutional systems + human systems = the intersection. The work fails when either side is ignored.</t>
+          <t>Every engagement leaves reusable knowledge, templates, and proof. We get stronger; clients get less dependent.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>9 · Nathan + Allie</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Institutional systems + human systems = the intersection. The work fails when either side is ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>10 · Next 12 months</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>A handful of warm wins, the Map as the first sale, Permit &amp; Bridge as the wedge. Modest and real.</t>
         </is>
@@ -936,7 +951,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -946,24 +961,24 @@
           <t>CMRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="21" t="n">
         <v>60000</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="22" t="n">
         <v>0.45</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="23">
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(E11)),D11*E11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -973,24 +988,24 @@
           <t>MRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="21" t="n">
         <v>50000</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="22" t="n">
         <v>0.4</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="23">
         <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),D12*E12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1000,24 +1015,24 @@
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="21" t="n">
         <v>35000</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="22" t="n">
         <v>0.6</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="23">
         <f>IF(AND(ISNUMBER(D13),ISNUMBER(E13)),D13*E13,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1027,24 +1042,24 @@
           <t>Existing network</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>Strongest</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="21" t="n">
         <v>25000</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="22" t="n">
         <v>0.65</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="23">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(E14)),D14*E14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1054,24 +1069,24 @@
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="21" t="n">
         <v>40000</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="23">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(E15)),D15*E15,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1081,24 +1096,24 @@
           <t>MVPC / other RPCs</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="21" t="n">
         <v>50000</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="22" t="n">
         <v>0.25</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="23">
         <f>IF(AND(ISNUMBER(D16),ISNUMBER(E16)),D16*E16,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1108,18 +1123,18 @@
           <t>Community Paradigm (municipal consulting)</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="21" t="n">
         <v>30000</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="22" t="n">
         <v>0.25</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="23">
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(E17)),D17*E17,0)</f>
         <v/>
       </c>
@@ -1147,10 +1162,10 @@
           <t>A known trigger: turnover, a stalled project, a funding deadline, a capacity gap.</t>
         </is>
       </c>
-      <c r="C20" s="23" t="n"/>
-      <c r="D20" s="23" t="n"/>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="25" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
@@ -1163,10 +1178,10 @@
           <t>Confirm authority, budget, and that it's a known problem we solve.</t>
         </is>
       </c>
-      <c r="C21" s="23" t="n"/>
-      <c r="D21" s="23" t="n"/>
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="24" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
+      <c r="F21" s="25" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
@@ -1179,10 +1194,10 @@
           <t>A paid Stewardship Map — the entry move.</t>
         </is>
       </c>
-      <c r="C22" s="23" t="n"/>
-      <c r="D22" s="23" t="n"/>
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="24" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
+      <c r="F22" s="25" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
@@ -1195,10 +1210,10 @@
           <t>Deliver the project, funding, permit, implementation, or capacity work.</t>
         </is>
       </c>
-      <c r="C23" s="23" t="n"/>
-      <c r="D23" s="23" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="24" t="n"/>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
+      <c r="F23" s="25" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -1211,10 +1226,10 @@
           <t>Transfer ownership; optional Implementation or Capacity Support.</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n"/>
-      <c r="D24" s="23" t="n"/>
-      <c r="E24" s="23" t="n"/>
-      <c r="F24" s="24" t="n"/>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="25" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
@@ -1227,10 +1242,10 @@
           <t>Capture the evidence — which becomes the next Signal.</t>
         </is>
       </c>
-      <c r="C25" s="23" t="n"/>
-      <c r="D25" s="23" t="n"/>
-      <c r="E25" s="23" t="n"/>
-      <c r="F25" s="24" t="n"/>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2027,7 +2042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2235,151 +2250,261 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>THE OFFER LADDER  —  free tier creates trust; paid tiers handle complexity</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Public Permit Helper / “Can I Do This?”</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Free or very low cost</t>
-        </is>
-      </c>
-    </row>
+          <t>THE FULL LADDER, FROM FREE TO WHITE-GLOVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>LogicCommons is the public access layer. It offers free templates, checklists, and simple frameworks that help residents, small organizations, and project sponsors understand the path before they need paid help.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>Permit Path Scan</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>$250 – $750</t>
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>PublicLogic piece</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Purpose</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Free public tools</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Stewardship Map</t>
+          <t>LogicCommons templates</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>$2,500 – $7,500</t>
+          <t>Help people self-serve basic planning, permit, grant, and project questions.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Cheap triage</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Permit &amp; Bridge Sprint</t>
+          <t>Permit Path Scan</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>$7,500 – $15,000</t>
+          <t>“What path am I probably on?”</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Paid diagnostic</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>White-Glove Implementation</t>
+          <t>Stewardship Map</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>$3,500 – $8,500 / month</t>
+          <t>“What actually needs to happen, who owns it, and what breaks?”</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>White-glove help</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Funding / Grant Build</t>
+          <t>Permit &amp; Bridge / Funding / Implementation</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>$5,000 – $25,000 (scope-dependent)</t>
+          <t>PublicLogic carries the project forward.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
+          <t>LogicCommons helps people start. PublicLogic helps them carry it through.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>THE OFFER LADDER  —  free tier creates trust; paid tiers handle complexity</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Public Permit Helper / “Can I Do This?”</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Free or very low cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Permit Path Scan</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>$250 – $750</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Stewardship Map</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>$2,500 – $7,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Permit &amp; Bridge Sprint</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>$7,500 – $15,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>White-Glove Implementation</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>$3,500 – $8,500 / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Funding / Grant Build</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>$5,000 – $25,000 (scope-dependent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="inlineStr">
+        <is>
           <t>Permit &amp; Bridge helps the public understand the path and helps project sponsors move through it.  That's the full product.</t>
         </is>
       </c>
     </row>
-    <row r="38"/>
+    <row r="49"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="15">
     <mergeCell ref="A16:C17"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A29:C30"/>
     <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A48:C49"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A25:C26"/>
+    <mergeCell ref="A39:C39"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A37:C38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2731,14 +2856,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>PublicLogic should be stronger after every engagement.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>The client should be less dependent after every engagement.</t>
         </is>

</xml_diff>

<commit_message>
Add credit policy: one tier's fee credits forward, no stacking
Both scope sheets (Stewardship Map, Permit Path Scan) and the workbook's
offer ladder now state the credit policy in plain language: a paid tier
credits toward the next engagement, but credits don't stack — up to one
tier's fee credits forward. Keeps entry risk low without eroding follow-on
margin.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -2042,7 +2042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2481,17 +2481,26 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="18" t="inlineStr">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>Credit policy: a paid tier credits toward the next engagement, but credits don't stack — up to one tier's fee credits forward. Keeps the entry risk low without eroding margin on a follow-on sprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge helps the public understand the path and helps project sponsors move through it.  That's the full product.</t>
         </is>
       </c>
     </row>
-    <row r="49"/>
+    <row r="51"/>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="A16:C17"/>
     <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A50:C51"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A29:C30"/>
     <mergeCell ref="A23:C23"/>

</xml_diff>

<commit_message>
Freeze workbook: LogicCommons box, P&B promise, stewardship-vs-consulting
Final three edits before freeze:
- Explicit LogicCommons box on Permit & Bridge (the public access layer,
  not a lead magnet): free templates/checklists/frameworks; "LogicCommons
  helps people start. PublicLogic helps them carry it through."
- Permit & Bridge promise: a sponsor leaves with a clear path forward, a
  clear record of how they got there, and a clear understanding of who
  owns what next.
- Transfer: "If neither happens, we are doing consulting instead of
  stewardship." — the philosophical center.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,6 +95,12 @@
     </font>
     <font>
       <b val="1"/>
+      <i val="1"/>
+      <color rgb="000F4C3A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -130,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -196,11 +202,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -234,6 +289,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -241,6 +306,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -250,9 +318,7 @@
     <xf numFmtId="9" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="14" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -951,7 +1017,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -961,24 +1027,24 @@
           <t>CMRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="30" t="n">
         <v>60000</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E11" s="31" t="n">
         <v>0.45</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="32">
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(E11)),D11*E11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -988,24 +1054,24 @@
           <t>MRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="29" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="30" t="n">
         <v>50000</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="31" t="n">
         <v>0.4</v>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="32">
         <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),D12*E12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1015,24 +1081,24 @@
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="30" t="n">
         <v>35000</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="31" t="n">
         <v>0.6</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="32">
         <f>IF(AND(ISNUMBER(D13),ISNUMBER(E13)),D13*E13,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1042,24 +1108,24 @@
           <t>Existing network</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="29" t="inlineStr">
         <is>
           <t>Strongest</t>
         </is>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="30" t="n">
         <v>25000</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="31" t="n">
         <v>0.65</v>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="32">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(E14)),D14*E14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1069,24 +1135,24 @@
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="30" t="n">
         <v>40000</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="31" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="23">
+      <c r="F15" s="32">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(E15)),D15*E15,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1096,24 +1162,24 @@
           <t>MVPC / other RPCs</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="30" t="n">
         <v>50000</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="31" t="n">
         <v>0.25</v>
       </c>
-      <c r="F16" s="23">
+      <c r="F16" s="32">
         <f>IF(AND(ISNUMBER(D16),ISNUMBER(E16)),D16*E16,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1123,18 +1189,18 @@
           <t>Community Paradigm (municipal consulting)</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="29" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="30" t="n">
         <v>30000</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="31" t="n">
         <v>0.25</v>
       </c>
-      <c r="F17" s="23">
+      <c r="F17" s="32">
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(E17)),D17*E17,0)</f>
         <v/>
       </c>
@@ -1162,10 +1228,10 @@
           <t>A known trigger: turnover, a stalled project, a funding deadline, a capacity gap.</t>
         </is>
       </c>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="25" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="18" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
@@ -1178,10 +1244,10 @@
           <t>Confirm authority, budget, and that it's a known problem we solve.</t>
         </is>
       </c>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="25" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="18" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
@@ -1194,10 +1260,10 @@
           <t>A paid Stewardship Map — the entry move.</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="25" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="18" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
@@ -1210,10 +1276,10 @@
           <t>Deliver the project, funding, permit, implementation, or capacity work.</t>
         </is>
       </c>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="25" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="18" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -1226,10 +1292,10 @@
           <t>Transfer ownership; optional Implementation or Capacity Support.</t>
         </is>
       </c>
-      <c r="C24" s="24" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="25" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="18" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
@@ -1242,10 +1308,10 @@
           <t>Capture the evidence — which becomes the next Signal.</t>
         </is>
       </c>
-      <c r="C25" s="24" t="n"/>
-      <c r="D25" s="24" t="n"/>
-      <c r="E25" s="24" t="n"/>
-      <c r="F25" s="25" t="n"/>
+      <c r="C25" s="17" t="n"/>
+      <c r="D25" s="17" t="n"/>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2042,7 +2108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2124,396 +2190,433 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>The promise</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>A project sponsor should leave with a clear path forward, a clear record of how they got there, and a clear understanding of who owns what next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>TWO SIDES OF THE SAME BRIDGE</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Layer</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Audience</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>Offer</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Public Help Layer</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Residents · small owners · nonprofits</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>“Can I do X in my backyard / property / building?”  Cheap, simple, framework-guided.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
+          <t>Public Help Layer</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Residents · small owners · nonprofits</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>“Can I do X in my backyard / property / building?”  Cheap, simple, framework-guided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
           <t>Project Sponsor Layer</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Developers · towns · nonprofits · businesses</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>White-glove permit path · stewardship map · grant / funding strategy · implementation support.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>LogicCommons — the public access layer</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="18" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Free templates, checklists, and frameworks that help people understand the path before they need paid help.   LogicCommons helps people start. PublicLogic helps them carry it through.</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="21" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="n"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="24" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>PERMIT &amp; BRIDGE: PUBLIC OUTPUT LAYER</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>The free/cheap tier is NOT AI consulting. It is a guided public framework that helps people understand the path. PublicLogic can support a simple public-facing assistance layer for common questions:</t>
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>•  “Can I put this in my backyard?”</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>•  “Do I need a permit?”</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>•  “Who do I ask first?”</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>•  “What board or office handles this?”</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>•  “What documents will I likely need?”</t>
-        </is>
-      </c>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
+          <t>•  “Can I put this in my backyard?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>•  “Do I need a permit?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>•  “Who do I ask first?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>•  “What board or office handles this?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>•  “What documents will I likely need?”</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t>•  “Is this a zoning, building, health, conservation, or licensing issue?”</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>This layer should be low-cost or free — its purpose is access, trust, and triage. It does NOT replace the municipality, inspector, planner, or permitting authority. It helps people ask better questions, gather the right information, and avoid wasting time.</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="31"/>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>THE FULL LADDER, FROM FREE TO WHITE-GLOVE</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>LogicCommons is the public access layer. It offers free templates, checklists, and simple frameworks that help residents, small organizations, and project sponsors understand the path before they need paid help.</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Layer</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>PublicLogic piece</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Free public tools</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>LogicCommons templates</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>Help people self-serve basic planning, permit, grant, and project questions.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>Cheap triage</t>
         </is>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Permit Path Scan</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>“What path am I probably on?”</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Paid diagnostic</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Stewardship Map</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>“What actually needs to happen, who owns it, and what breaks?”</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>White-glove help</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge / Funding / Implementation</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>PublicLogic carries the project forward.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>LogicCommons helps people start. PublicLogic helps them carry it through.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>THE OFFER LADDER  —  free tier creates trust; paid tiers handle complexity</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
         <is>
           <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>Public Permit Helper / “Can I Do This?”</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>Free or very low cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="inlineStr">
-        <is>
-          <t>Permit Path Scan</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>$250 – $750</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Stewardship Map</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>$2,500 – $7,500</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>Permit &amp; Bridge Sprint</t>
-        </is>
-      </c>
-      <c r="C44" s="11" t="inlineStr">
-        <is>
-          <t>$7,500 – $15,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>White-Glove Implementation</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>$3,500 – $8,500 / month</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Public Permit Helper / “Can I Do This?”</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Free or very low cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>Permit Path Scan</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>$250 – $750</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Stewardship Map</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>$2,500 – $7,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Permit &amp; Bridge Sprint</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>$7,500 – $15,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>White-Glove Implementation</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>$3,500 – $8,500 / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>Funding / Grant Build</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>$5,000 – $25,000 (scope-dependent)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>Credit policy: a paid tier credits toward the next engagement, but credits don't stack — up to one tier's fee credits forward. Keeps the entry risk low without eroding margin on a follow-on sprint.</t>
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50">
-      <c r="A50" s="18" t="inlineStr">
+    <row r="54"/>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge helps the public understand the path and helps project sponsors move through it.  That's the full product.</t>
         </is>
       </c>
     </row>
-    <row r="51"/>
+    <row r="56"/>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A16:C17"/>
+  <mergeCells count="18">
+    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A50:C51"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A29:C30"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A21:C22"/>
     <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A48:C49"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A30:C31"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A53:C54"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A17:C18"/>
+    <mergeCell ref="A34:C35"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A55:C56"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2865,16 +2968,23 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>PublicLogic should be stronger after every engagement.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>The client should be less dependent after every engagement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>If neither happens, we are doing consulting instead of stewardship.</t>
         </is>
       </c>
     </row>
@@ -2887,8 +2997,9 @@
     </row>
     <row r="14"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A13:B14"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Name the delivery infrastructure: Continuity System
Replace the techy "carriers" framing with a plain-English umbrella term
clients can actually say. "Continuity System" = PublicLogic's delivery
infrastructure (CaseSpaces, VAULT, PuddleJumper, Workbooks/Registers/
Templates, with LogicCommons as the public version). It answers the only
question a buyer asks: "If my planner leaves, does this still work?"

- Start Here: the four-layer architecture (LogicCommons = public access ·
  Permit & Bridge = navigation · PublicLogic = services · Continuity System
  = delivery infrastructure).
- Transfer: reframed the components as the Continuity System.
"The Chair" stays as philosophy only, not a product term.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -756,118 +756,130 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>1 · Why we exist</t>
+          <t>The architecture</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Good work keeps failing when knowledge, ownership, or continuity disappears. We've watched it happen, and we built the practices to stop it.</t>
+          <t>LogicCommons = public access layer · Permit &amp; Bridge = navigation layer · PublicLogic = services · Continuity System = delivery infrastructure.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2 · The problem</t>
+          <t>1 · Why we exist</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Capacity stops keeping pace with complexity. The 'Chair' — the place where a function lives — ends up depending on one person.</t>
+          <t>Good work keeps failing when knowledge, ownership, or continuity disappears. We've watched it happen, and we built the practices to stop it.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>3 · What clients buy</t>
+          <t>2 · The problem</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Projects moved forward. Funding found and won. A role or function covered.</t>
+          <t>Capacity stops keeping pace with complexity. The 'Chair' — the place where a function lives — ends up depending on one person.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>4 · What we deliver</t>
+          <t>3 · What clients buy</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>The same — plus the stewardship that makes it survive turnover.</t>
+          <t>Projects moved forward. Funding found and won. A role or function covered.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>5 · What makes us different</t>
+          <t>4 · What we deliver</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Most systems manage work. PublicLogic helps steward what has to survive the work.</t>
+          <t>The same — plus the stewardship that makes it survive turnover.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>6 · What we sell</t>
+          <t>5 · What makes us different</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Stewardship Map (the safe first step) → Sprints (Project · Funding · Permit &amp; Bridge) → Implementation &amp; Capacity Support.</t>
+          <t>Most systems manage work. PublicLogic helps steward what has to survive the work.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>7 · Who first</t>
+          <t>6 · What we sell</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Our existing municipal network, regional planning agencies, engineering firms, municipal consulting firms.</t>
+          <t>Stewardship Map (the safe first step) → Sprints (Project · Funding · Permit &amp; Bridge) → Implementation &amp; Capacity Support.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>8 · How it compounds</t>
+          <t>7 · Who first</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Every engagement leaves reusable knowledge, templates, and proof. We get stronger; clients get less dependent.</t>
+          <t>Our existing municipal network, regional planning agencies, engineering firms, municipal consulting firms.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>9 · Nathan + Allie</t>
+          <t>8 · How it compounds</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Institutional systems + human systems = the intersection. The work fails when either side is ignored.</t>
+          <t>Every engagement leaves reusable knowledge, templates, and proof. We get stronger; clients get less dependent.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>9 · Nathan + Allie</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Institutional systems + human systems = the intersection. The work fails when either side is ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>10 · Next 12 months</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>A handful of warm wins, the Map as the first sale, Permit &amp; Bridge as the wedge. Modest and real.</t>
         </is>
@@ -2879,7 +2891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2988,17 +3000,34 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>The carriers (plain language):  LogicCommons — shared templates &amp; frameworks.   CaseSpaces — a project's governed record.   PuddleJumper — the workflow/process layer.   VAULT — how knowledge is preserved so it survives turnover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>THE CONTINUITY SYSTEM — our delivery infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="56" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Every engagement is delivered through a Continuity System: the records, decisions, templates, and processes that keep the work alive after we step back. In plain language —  CaseSpaces: a project's governed record.   VAULT: how knowledge is preserved so it survives turnover.   PuddleJumper: the workflow/process layer.   Workbooks · Registers · Templates: the reusable artifacts.   LogicCommons: the public, free version of the same templates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>A client never has to care about VAULT or CaseSpaces. They care about one thing: “If my planner leaves, does this still work?” A Continuity System is how we answer yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A13:B14"/>
+  <mergeCells count="4">
+    <mergeCell ref="A15:B16"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Clarify: PuddleJumper IS the Continuity System
PuddleJumper is the name of the delivery infrastructure, not a peer
component. "Continuity System" is the plain-English category we say to a
client; PuddleJumper is what we call it. CaseSpaces (governed record),
VAULT (knowledge preservation), and Workbooks/Registers/Templates are
components inside it. LogicCommons is explicitly separate — the public
free layer, not part of a client's Continuity System.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +98,10 @@
       <i val="1"/>
       <color rgb="000F4C3A"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="006B6660"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -255,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -309,6 +313,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -318,7 +325,7 @@
     <xf numFmtId="9" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="15" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -761,7 +768,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>LogicCommons = public access layer · Permit &amp; Bridge = navigation layer · PublicLogic = services · Continuity System = delivery infrastructure.</t>
+          <t>LogicCommons = public access layer · Permit &amp; Bridge = navigation layer · PublicLogic = services · Continuity System (PuddleJumper) = delivery infrastructure.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1036,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1039,24 +1046,24 @@
           <t>CMRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D11" s="30" t="n">
+      <c r="D11" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="E11" s="31" t="n">
+      <c r="E11" s="32" t="n">
         <v>0.45</v>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="33">
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(E11)),D11*E11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1066,24 +1073,24 @@
           <t>MRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="30" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="31" t="n">
         <v>50000</v>
       </c>
-      <c r="E12" s="31" t="n">
+      <c r="E12" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="33">
         <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),D12*E12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1093,24 +1100,24 @@
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="D13" s="30" t="n">
+      <c r="D13" s="31" t="n">
         <v>35000</v>
       </c>
-      <c r="E13" s="31" t="n">
+      <c r="E13" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="33">
         <f>IF(AND(ISNUMBER(D13),ISNUMBER(E13)),D13*E13,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1120,24 +1127,24 @@
           <t>Existing network</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="30" t="inlineStr">
         <is>
           <t>Strongest</t>
         </is>
       </c>
-      <c r="D14" s="30" t="n">
+      <c r="D14" s="31" t="n">
         <v>25000</v>
       </c>
-      <c r="E14" s="31" t="n">
+      <c r="E14" s="32" t="n">
         <v>0.65</v>
       </c>
-      <c r="F14" s="32">
+      <c r="F14" s="33">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(E14)),D14*E14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1147,24 +1154,24 @@
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D15" s="30" t="n">
+      <c r="D15" s="31" t="n">
         <v>40000</v>
       </c>
-      <c r="E15" s="31" t="n">
+      <c r="E15" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="32">
+      <c r="F15" s="33">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(E15)),D15*E15,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1174,24 +1181,24 @@
           <t>MVPC / other RPCs</t>
         </is>
       </c>
-      <c r="C16" s="29" t="inlineStr">
+      <c r="C16" s="30" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D16" s="30" t="n">
+      <c r="D16" s="31" t="n">
         <v>50000</v>
       </c>
-      <c r="E16" s="31" t="n">
+      <c r="E16" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="33">
         <f>IF(AND(ISNUMBER(D16),ISNUMBER(E16)),D16*E16,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1201,18 +1208,18 @@
           <t>Community Paradigm (municipal consulting)</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="30" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D17" s="30" t="n">
+      <c r="D17" s="31" t="n">
         <v>30000</v>
       </c>
-      <c r="E17" s="31" t="n">
+      <c r="E17" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="F17" s="32">
+      <c r="F17" s="33">
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(E17)),D17*E17,0)</f>
         <v/>
       </c>
@@ -2891,7 +2898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3003,31 +3010,39 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>THE CONTINUITY SYSTEM — our delivery infrastructure</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="56" customHeight="1">
+          <t>THE CONTINUITY SYSTEM — our delivery infrastructure (PuddleJumper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Every engagement is delivered through a Continuity System: the records, decisions, templates, and processes that keep the work alive after we step back. In plain language —  CaseSpaces: a project's governed record.   VAULT: how knowledge is preserved so it survives turnover.   PuddleJumper: the workflow/process layer.   Workbooks · Registers · Templates: the reusable artifacts.   LogicCommons: the public, free version of the same templates.</t>
+          <t>Every engagement is delivered through a Continuity System — the records, decisions, templates, and processes that keep the work alive after we step back. PuddleJumper is the name of that system. Inside it —  CaseSpaces: a project's governed record.   VAULT: how knowledge is preserved so it survives turnover.   Workbooks · Registers · Templates: the reusable artifacts the work runs on.  ('Continuity System' is what we say to a client; 'PuddleJumper' is what we call it.)</t>
         </is>
       </c>
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>A client never has to care about VAULT or CaseSpaces. They care about one thing: “If my planner leaves, does this still work?” A Continuity System is how we answer yes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>LogicCommons is separate — the public, free layer (templates for residents and sponsors), not part of a client's Continuity System.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>A client never has to care about CaseSpaces or VAULT. They care about one thing: “If my planner leaves, does this still work?” A Continuity System is how we answer yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A15:B16"/>
-    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="A18:B19"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adopt "Continuity & Stewardship Systems" as the delivery category
Elevate the delivery infrastructure to a phrase that reads like a real
company and doesn't sound like software: Continuity (the outcome) +
Stewardship (the practice) + Systems (the mechanism).

- What We Do: "PublicLogic provides project development, funding strategy,
  implementation support, and capacity support through Continuity &
  Stewardship Systems."
- Transfer: "How We Deliver" — the definition, the "may include" component
  list (CaseSpaces, Workbooks, Registers, Templates, VAULT records,
  accountability structures, continuity plans, project environments, proof
  frameworks). PuddleJumper named only as the under-the-hood layer; goal is
  always "make it easier for the next person to do the right thing."
- Start Here architecture line updated to match.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +98,11 @@
       <i val="1"/>
       <color rgb="000F4C3A"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F4C3A"/>
+      <sz val="10"/>
     </font>
     <font>
       <color rgb="006B6660"/>
@@ -259,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -313,7 +318,8 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -325,7 +331,7 @@
     <xf numFmtId="9" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="16" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -768,7 +774,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>LogicCommons = public access layer · Permit &amp; Bridge = navigation layer · PublicLogic = services · Continuity System (PuddleJumper) = delivery infrastructure.</t>
+          <t>LogicCommons = public access layer · Permit &amp; Bridge = navigation layer · PublicLogic = services · Continuity &amp; Stewardship Systems = how we deliver (records, processes, templates, environments, accountability).</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1042,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1046,24 +1052,24 @@
           <t>CMRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C11" s="30" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D11" s="31" t="n">
+      <c r="D11" s="32" t="n">
         <v>60000</v>
       </c>
-      <c r="E11" s="32" t="n">
+      <c r="E11" s="33" t="n">
         <v>0.45</v>
       </c>
-      <c r="F11" s="33">
+      <c r="F11" s="34">
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(E11)),D11*E11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1073,24 +1079,24 @@
           <t>MRPC (regional planning)</t>
         </is>
       </c>
-      <c r="C12" s="30" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="32" t="n">
         <v>50000</v>
       </c>
-      <c r="E12" s="32" t="n">
+      <c r="E12" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="F12" s="33">
+      <c r="F12" s="34">
         <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),D12*E12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1100,24 +1106,24 @@
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="D13" s="31" t="n">
+      <c r="D13" s="32" t="n">
         <v>35000</v>
       </c>
-      <c r="E13" s="32" t="n">
+      <c r="E13" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="34">
         <f>IF(AND(ISNUMBER(D13),ISNUMBER(E13)),D13*E13,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1127,24 +1133,24 @@
           <t>Existing network</t>
         </is>
       </c>
-      <c r="C14" s="30" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>Strongest</t>
         </is>
       </c>
-      <c r="D14" s="31" t="n">
+      <c r="D14" s="32" t="n">
         <v>25000</v>
       </c>
-      <c r="E14" s="32" t="n">
+      <c r="E14" s="33" t="n">
         <v>0.65</v>
       </c>
-      <c r="F14" s="33">
+      <c r="F14" s="34">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(E14)),D14*E14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
@@ -1154,24 +1160,24 @@
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
+      <c r="C15" s="31" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D15" s="31" t="n">
+      <c r="D15" s="32" t="n">
         <v>40000</v>
       </c>
-      <c r="E15" s="32" t="n">
+      <c r="E15" s="33" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="33">
+      <c r="F15" s="34">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(E15)),D15*E15,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1181,24 +1187,24 @@
           <t>MVPC / other RPCs</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D16" s="31" t="n">
+      <c r="D16" s="32" t="n">
         <v>50000</v>
       </c>
-      <c r="E16" s="32" t="n">
+      <c r="E16" s="33" t="n">
         <v>0.25</v>
       </c>
-      <c r="F16" s="33">
+      <c r="F16" s="34">
         <f>IF(AND(ISNUMBER(D16),ISNUMBER(E16)),D16*E16,0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Qualify</t>
         </is>
@@ -1208,18 +1214,18 @@
           <t>Community Paradigm (municipal consulting)</t>
         </is>
       </c>
-      <c r="C17" s="30" t="inlineStr">
+      <c r="C17" s="31" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D17" s="31" t="n">
+      <c r="D17" s="32" t="n">
         <v>30000</v>
       </c>
-      <c r="E17" s="32" t="n">
+      <c r="E17" s="33" t="n">
         <v>0.25</v>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="34">
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(E17)),D17*E17,0)</f>
         <v/>
       </c>
@@ -1712,7 +1718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1786,87 +1792,99 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>How we deliver</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>PublicLogic provides project development, funding strategy, implementation support, and capacity support through Continuity &amp; Stewardship Systems — the records, processes, templates, environments, and accountability structures that help important work survive turnover and change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>THE EQUATION</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Recommended (use this one):  Good Work + Stewardship = Work That Lasts</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Fuller / operational:  Project + Funding + Capacity + Continuity = Implementation</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="14" t="inlineStr">
         <is>
+          <t>Fuller / operational:  Project + Funding + Capacity + Continuity = Implementation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
           <t>Fuller / outcomes:  Vision + Funding + Capacity + Stewardship = Durable Results</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>HOW WE WORK</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Map  →  Embed  →  Encode  →  Sustain</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Map</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Surface how work, knowledge, authority, records, and risk actually move.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Embed</t>
+          <t>Map</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Put the right structure into the live workflow, with the people who do the work.</t>
+          <t>Surface how work, knowledge, authority, records, and risk actually move.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Encode</t>
+          <t>Embed</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Capture the knowledge and rules so they outlast any individual.</t>
+          <t>Put the right structure into the live workflow, with the people who do the work.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Capture the knowledge and rules so they outlast any individual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
           <t>Sustain</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Monitor adoption and transfer ownership so it runs without us.</t>
         </is>
@@ -2898,7 +2916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3010,39 +3028,57 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>THE CONTINUITY SYSTEM — our delivery infrastructure (PuddleJumper)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+          <t>HOW WE DELIVER — Continuity &amp; Stewardship Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Every engagement is delivered through a Continuity System — the records, decisions, templates, and processes that keep the work alive after we step back. PuddleJumper is the name of that system. Inside it —  CaseSpaces: a project's governed record.   VAULT: how knowledge is preserved so it survives turnover.   Workbooks · Registers · Templates: the reusable artifacts the work runs on.  ('Continuity System' is what we say to a client; 'PuddleJumper' is what we call it.)</t>
+          <t>The records, processes, templates, environments, and accountability structures that help important work survive turnover, changing priorities, and organizational change.   Continuity = the outcome.  Stewardship = the practice.  Systems = the mechanism.</t>
         </is>
       </c>
     </row>
     <row r="16"/>
-    <row r="17">
-      <c r="A17" s="29" t="inlineStr">
-        <is>
-          <t>LogicCommons is separate — the public, free layer (templates for residents and sponsors), not part of a client's Continuity System.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>A client never has to care about CaseSpaces or VAULT. They care about one thing: “If my planner leaves, does this still work?” A Continuity System is how we answer yes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>PublicLogic engagements create Continuity &amp; Stewardship Systems tailored to the project, organization, or initiative. The exact components vary; the goal is always the same — make it easier for the next person to do the right thing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>May include:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>CaseSpaces · Workbooks · Registers · Templates · VAULT records · Accountability structures · Continuity plans · Project environments · Proof frameworks.   (Under the hood these run on PuddleJumper — no one needs that name unless they want to go deeper. LogicCommons is the separate public, free layer.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>A client never has to care about the components. They care about one thing: “If my planner leaves, does this still work?” A Continuity &amp; Stewardship System is how we answer yes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="A22:B23"/>
+    <mergeCell ref="A20:B21"/>
     <mergeCell ref="A15:B16"/>
-    <mergeCell ref="A18:B19"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A17:B18"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Final adds: "How the Pieces Fit Together" table + tighten C&S Systems
- Start Here: a buyer's-eye routing table — "If you say... start here":
  template -> LogicCommons; question/navigate -> Permit & Bridge; have a
  project -> Stewardship Map; need it done -> PublicLogic. The single most
  useful thing for a website visitor.
- Continuity & Stewardship Systems: short mention in What We Do ("designed
  to preserve knowledge, accountability, continuity, and momentum"),
  defined in full once on Transfer (now includes "and proof"). It's the
  plumbing, not a product.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -56,13 +56,13 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001A1D20"/>
-      <sz val="15"/>
+      <color rgb="000F4C3A"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000F4C3A"/>
-      <sz val="12"/>
+      <color rgb="001A1D20"/>
+      <sz val="15"/>
     </font>
     <font>
       <i val="1"/>
@@ -275,20 +275,20 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -308,7 +308,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -697,10 +697,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="104" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -898,7 +898,77 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>HOW THE PIECES FIT TOGETHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>If you say…</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>…start here</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>“I need a template.”</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>LogicCommons</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>“I have a question / how do I navigate this?”</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Permit &amp; Bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>“I have a project — what actually needs to happen?”</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Stewardship Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>“I need help getting this done.”</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>PublicLogic (Sprints · Implementation · Capacity)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A20:B20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -921,7 +991,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Who We Pursue — Forced Prioritization</t>
         </is>
@@ -935,107 +1005,107 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Pursue</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Tier 1 — now</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Existing municipal network · Regional planning agencies · Engineering firms · Municipal consulting firms</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Already have projects and budgets; warmest relationships; shortest sales cycle.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Tier 2 — next</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Developers · Housing organizations · Community development organizations</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Real need (especially Permit &amp; Bridge), longer cycle; pursue once Tier 1 is producing.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Tier 3 — later</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Everything else</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Interesting, but not now. Don't chase.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>TIER-1 PIPELINE  (illustrative Revenue/Probability — replace with real figures; Weighted = Revenue x Probability; sort to rank)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Pursue</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Relationship</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Weighted ($)</t>
         </is>
@@ -1047,7 +1117,7 @@
           <t>NOW</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>CMRPC (regional planning)</t>
         </is>
@@ -1074,7 +1144,7 @@
           <t>NOW</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>MRPC (regional planning)</t>
         </is>
@@ -1101,7 +1171,7 @@
           <t>NOW</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
@@ -1128,7 +1198,7 @@
           <t>NOW</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Existing network</t>
         </is>
@@ -1155,7 +1225,7 @@
           <t>NOW</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
@@ -1182,7 +1252,7 @@
           <t>Qualify</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>MVPC / other RPCs</t>
         </is>
@@ -1209,7 +1279,7 @@
           <t>Qualify</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Community Paradigm (municipal consulting)</t>
         </is>
@@ -1231,7 +1301,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>ENGAGEMENT FLOW</t>
         </is>
@@ -1248,7 +1318,7 @@
           <t>Signal</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>A known trigger: turnover, a stalled project, a funding deadline, a capacity gap.</t>
         </is>
@@ -1264,7 +1334,7 @@
           <t>Fit</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Confirm authority, budget, and that it's a known problem we solve.</t>
         </is>
@@ -1280,7 +1350,7 @@
           <t>Map</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>A paid Stewardship Map — the entry move.</t>
         </is>
@@ -1296,7 +1366,7 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Deliver the project, funding, permit, implementation, or capacity work.</t>
         </is>
@@ -1312,7 +1382,7 @@
           <t>Sustain</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Transfer ownership; optional Implementation or Capacity Support.</t>
         </is>
@@ -1328,7 +1398,7 @@
           <t>Prove</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Capture the evidence — which becomes the next Signal.</t>
         </is>
@@ -1367,7 +1437,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>What's Realistic in the Next 12 Months</t>
         </is>
@@ -1381,95 +1451,95 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>The honest goal for year one is not scale. It's a small number of real, paid engagements with people who already trust us — and a repeatable way to do them.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr"/>
+      <c r="A5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Move</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>What it looks like</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Sell a few Maps</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>2–4 paid Stewardship Maps with warm Tier-1 relationships.</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Low-risk entry; surfaces the next, bigger engagement; builds reference proof.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Convert 1–2</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Turn a Map into Project / Funding / Permit &amp; Bridge work.</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>This is where the real revenue is, and where Permit &amp; Bridge proves out.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Land baseline retainers</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>1–2 monthly Implementation or Capacity engagements.</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Predictable monthly revenue that smooths the project lumpiness.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Build the templates as we go</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Every engagement leaves a reusable asset (Transfer tab).</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Each job gets cheaper to deliver; we compound instead of resetting.</t>
         </is>
@@ -1504,7 +1574,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Why PublicLogic Exists</t>
         </is>
@@ -1518,51 +1588,51 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>PublicLogic came out of real work — Hubbardston, Sutton, Phillipston, Gardiner, Michigan LTC — and out of years inside municipal administration, capital planning, and grant development.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr"/>
+      <c r="A5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Across all of it we kept seeing the same thing: good, important work would stall or quietly disappear. Not because the idea was wrong. Because the person holding it left, the knowledge was never written down, or no one owned what came next.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr"/>
+      <c r="A7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>PublicLogic is our attempt to fix that — with the practices we wish we'd had when we were inside it.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
+      <c r="A9" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>North Star</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>“Every system should make it easier for the next person to do the right thing.”</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>This isn't a new company we're inventing. It's the company that already exists — named, and made repeatable.</t>
         </is>
@@ -1587,7 +1657,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>What Breaks Without Stewardship</t>
         </is>
@@ -1601,96 +1671,96 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>When stewardship is missing…</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>…this is what we've watched happen</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Turnover</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>The person leaves and the knowledge leaves with them.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Lost knowledge</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>How and why things were done stops being written down.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Delayed projects</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Work stalls because no one owns the next step.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Missed funding</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>A funding window closes before anyone is ready.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Dependency on individuals</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>The whole function runs through one person's head.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Repeated mistakes</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>The same problems come back because nothing was captured.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Plans that never become action</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>A good plan gets made, then sits on a shelf.</t>
         </is>
@@ -1726,7 +1796,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>What PublicLogic Actually Does</t>
         </is>
@@ -1800,12 +1870,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>PublicLogic provides project development, funding strategy, implementation support, and capacity support through Continuity &amp; Stewardship Systems — the records, processes, templates, environments, and accountability structures that help important work survive turnover and change.</t>
+          <t>PublicLogic delivers services through Continuity &amp; Stewardship Systems designed to preserve knowledge, accountability, continuity, and momentum. (Defined once on the Transfer tab — it's the plumbing, not a product.)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>THE EQUATION</t>
         </is>
@@ -1831,7 +1901,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>HOW WE WORK</t>
         </is>
@@ -1848,7 +1918,7 @@
           <t>Map</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Surface how work, knowledge, authority, records, and risk actually move.</t>
         </is>
@@ -1860,7 +1930,7 @@
           <t>Embed</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Put the right structure into the live workflow, with the people who do the work.</t>
         </is>
@@ -1872,7 +1942,7 @@
           <t>Encode</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Capture the knowledge and rules so they outlast any individual.</t>
         </is>
@@ -1884,7 +1954,7 @@
           <t>Sustain</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Monitor adoption and transfer ownership so it runs without us.</t>
         </is>
@@ -1912,7 +1982,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>The Offer Stack</t>
         </is>
@@ -1926,189 +1996,189 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Why it exists</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Transfer asset</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Stewardship Map  (entry)</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Understand how work, knowledge, authority, records, and risk actually move — before anyone commits money. The safest first engagement.</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Stewardship Map · Continuity Risks · Readiness Findings · Priority Roadmap</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>$2,500 – $7,500</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>CaseSpace + the Map</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Project Development Sprint</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Turn a priority or a challenge into an actionable project.</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Project Development Roadmap</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>$5,000 – $15,000</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Charter / Scope template</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Funding Strategy Sprint</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Find realistic funding and the readiness it requires.</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Funding Roadmap</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>$5,000 – $12,500</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Funding scan + roadmap workbook</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge Sprint</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Move a project through the public systems around it (permits, boards, funding, stakeholders).</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Approvals path + coordination plan</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>$7,500 – $15,000</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Bridge map / permit register</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Implementation Support</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Coordinate and hold accountability while a plan gets executed by the client's team.</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Implementation Framework + Accountability Structure</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>$3,500 – $8,500 / month</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>VAULT continuity record</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Capacity Support</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Step in and hold a role or function directly — interim / fractional — until it transfers back.</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Embedded Capacity Plan + Continuity Handoff</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>$4,000 – $10,000 / month</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Role / Coverage Map + handoff</t>
         </is>
@@ -2154,7 +2224,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge</t>
         </is>
@@ -2240,58 +2310,58 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>TWO SIDES OF THE SAME BRIDGE</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Layer</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Audience</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Offer</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Public Help Layer</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Residents · small owners · nonprofits</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>“Can I do X in my backyard / property / building?”  Cheap, simple, framework-guided.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Project Sponsor Layer</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Developers · towns · nonprofits · businesses</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>White-glove permit path · stewardship map · grant / funding strategy · implementation support.</t>
         </is>
@@ -2321,14 +2391,14 @@
       <c r="C18" s="24" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>PERMIT &amp; BRIDGE: PUBLIC OUTPUT LAYER</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>The free/cheap tier is NOT AI consulting. It is a guided public framework that helps people understand the path. PublicLogic can support a simple public-facing assistance layer for common questions:</t>
         </is>
@@ -2336,42 +2406,42 @@
     </row>
     <row r="22"/>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>•  “Can I put this in my backyard?”</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>•  “Do I need a permit?”</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>•  “Who do I ask first?”</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>•  “What board or office handles this?”</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>•  “What documents will I likely need?”</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>•  “Is this a zoning, building, health, conservation, or licensing issue?”</t>
         </is>
@@ -2386,14 +2456,14 @@
     </row>
     <row r="31"/>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>THE FULL LADDER, FROM FREE TO WHITE-GLOVE</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>LogicCommons is the public access layer. It offers free templates, checklists, and simple frameworks that help residents, small organizations, and project sponsors understand the path before they need paid help.</t>
         </is>
@@ -2401,85 +2471,85 @@
     </row>
     <row r="35"/>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Layer</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>PublicLogic piece</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>Free public tools</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>LogicCommons templates</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Help people self-serve basic planning, permit, grant, and project questions.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>Cheap triage</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>Permit Path Scan</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>“What path am I probably on?”</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>Paid diagnostic</t>
         </is>
       </c>
-      <c r="B39" s="11" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>Stewardship Map</t>
         </is>
       </c>
-      <c r="C39" s="11" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>“What actually needs to happen, who owns it, and what breaks?”</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>White-glove help</t>
         </is>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge / Funding / Implementation</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>PublicLogic carries the project forward.</t>
         </is>
@@ -2493,126 +2563,126 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>THE OFFER LADDER  —  free tier creates trust; paid tiers handle complexity</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>Public Permit Helper / “Can I Do This?”</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>Free or very low cost</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Permit Path Scan</t>
         </is>
       </c>
-      <c r="C47" s="11" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>$250 – $750</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>Stewardship Map</t>
         </is>
       </c>
-      <c r="C48" s="11" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>$2,500 – $7,500</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>Permit &amp; Bridge Sprint</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>$7,500 – $15,000</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>White-Glove Implementation</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>$3,500 – $8,500 / month</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B51" s="11" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>Funding / Grant Build</t>
         </is>
       </c>
-      <c r="C51" s="11" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>$5,000 – $25,000 (scope-dependent)</t>
         </is>
@@ -2675,7 +2745,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Proof — We Can Show It</t>
         </is>
@@ -2689,132 +2759,132 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Proof</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>What it shows</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>How we show it</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Continuity</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>A function survives when the person who ran it leaves.</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Successor test + structure mapped to authority and stop-rules.</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Sutton — the 30-day successor test the town would otherwise fail.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Record</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Every claim, number, and decision traces to a source.</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>A governed record: source file → workbook row → output.</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Michigan LTC corridor record — line-for-line traceability.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Readiness</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>The organization can absorb and sustain the change.</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Readiness findings in the Map, before any build.</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Pre-build assessment that sequences what the org can carry.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Adoption</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Staff actually use the system — not just receive it.</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Adoption monitoring through implementation (Allie's work).</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Shrewsbury — human-systems support so the build is used.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>The work moved forward and got funded.</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Funded applications and delivered projects, documented.</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Shrewsbury fiber, Sutton — funding secured, projects implemented.</t>
         </is>
@@ -2850,7 +2920,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Why We're Better Together</t>
         </is>
@@ -2867,7 +2937,7 @@
           <t>How municipalities, money, grants, procurement, and projects actually work — from the inside.</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr"/>
+      <c r="C4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -2924,7 +2994,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Transfer — Every Engagement Leaves Something Behind</t>
         </is>
@@ -2938,67 +3008,67 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Every engagement creates…</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Reusable knowledge</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>What we learned about how this kind of organization works.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Reusable templates</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Charters, roadmaps, registers, and workbooks we can adapt next time.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Reusable process</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>A repeatable way of doing the work — not a one-off.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Reusable proof</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Evidence (continuity / record / readiness / adoption / outcome) we can show the next client.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Two tests for every engagement:</t>
         </is>
@@ -3026,22 +3096,22 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>HOW WE DELIVER — Continuity &amp; Stewardship Systems</t>
         </is>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>The records, processes, templates, environments, and accountability structures that help important work survive turnover, changing priorities, and organizational change.   Continuity = the outcome.  Stewardship = the practice.  Systems = the mechanism.</t>
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>The records, processes, templates, environments, accountability structures, and proof needed to help important work survive turnover, changing priorities, and organizational change.   Continuity = the outcome.  Stewardship = the practice.  Systems = the mechanism.</t>
         </is>
       </c>
     </row>
     <row r="16"/>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>PublicLogic engagements create Continuity &amp; Stewardship Systems tailored to the project, organization, or initiative. The exact components vary; the goal is always the same — make it easier for the next person to do the right thing.</t>
         </is>

</xml_diff>

<commit_message>
Pipeline: drop dollars for Next Action; add "return to problem" + 5th verb
- Who We Pursue: remove revenue/weighted-value estimates (false precision)
  in favor of Target · Relationship · Probability · Next Action.
- Language tab: add "always return to the problem" guardrail — never use
  Institutional Stewardship by itself; tie it to turnover, lost knowledge,
  stalled projects, missed opportunities.
- Five layers, five verbs: Understand · Navigate · Diagnose · Deliver ·
  Sustain. Start Here architecture line + The Path foundation bar updated.
Refresh the v1 stack zip.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,9 +113,6 @@
     <font>
       <color rgb="006B6660"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <i val="1"/>
@@ -275,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -343,14 +340,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -795,7 +785,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>LogicCommons = public access layer · Permit &amp; Bridge = navigation layer · PublicLogic = services · Continuity &amp; Stewardship Systems = how we deliver (records, processes, templates, environments, accountability).</t>
+          <t>Five layers, five verbs:  LogicCommons = Understand · Permit &amp; Bridge = Navigate · Stewardship Map = Diagnose · PublicLogic = Deliver · Continuity &amp; Stewardship Systems = Sustain.</t>
         </is>
       </c>
     </row>
@@ -1003,12 +993,10 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1096,229 +1084,184 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>TIER-1 PIPELINE  (illustrative Revenue/Probability — replace with real figures; Weighted = Revenue x Probability; sort to rank)</t>
+          <t>TIER-1 PIPELINE  (no revenue estimates until they're real — track relationship, probability, and the next action)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Pursue</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Relationship</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Relationship</t>
+          <t>Probability</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Revenue ($)</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Probability</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Weighted ($)</t>
+          <t>Next action</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="34" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>CMRPC (regional planning)</t>
         </is>
       </c>
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>Developing</t>
+        </is>
+      </c>
       <c r="C11" s="34" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>Book an intro call; offer a paid Stewardship Map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>MRPC (regional planning)</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="inlineStr">
+        <is>
           <t>Developing</t>
         </is>
       </c>
-      <c r="D11" s="35" t="n">
-        <v>60000</v>
-      </c>
-      <c r="E11" s="36" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="F11" s="37">
-        <f>IF(AND(ISNUMBER(D11),ISNUMBER(E11)),D11*E11,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>MRPC (regional planning)</t>
-        </is>
-      </c>
       <c r="C12" s="34" t="inlineStr">
         <is>
-          <t>Developing</t>
-        </is>
-      </c>
-      <c r="D12" s="35" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E12" s="36" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F12" s="37">
-        <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),D12*E12,0)</f>
-        <v/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>Warm intro; share the one-pager.</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="34" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Warm municipal relationships (Sutton/Shrewsbury/Phillipston)</t>
         </is>
       </c>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
       <c r="C13" s="34" t="inlineStr">
         <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="D13" s="35" t="n">
-        <v>35000</v>
-      </c>
-      <c r="E13" s="36" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F13" s="37">
-        <f>IF(AND(ISNUMBER(D13),ISNUMBER(E13)),D13*E13,0)</f>
-        <v/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
+        <is>
+          <t>Propose a Map on a known stalled function.</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Existing network</t>
         </is>
       </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>Strongest</t>
+        </is>
+      </c>
       <c r="C14" s="34" t="inlineStr">
         <is>
-          <t>Strongest</t>
-        </is>
-      </c>
-      <c r="D14" s="35" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E14" s="36" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F14" s="37">
-        <f>IF(AND(ISNUMBER(D14),ISNUMBER(E14)),D14*E14,0)</f>
-        <v/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>Ask directly who needs a Map first.</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="34" t="inlineStr">
-        <is>
-          <t>NOW</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Fuss &amp; O'Neill (engineering)</t>
         </is>
       </c>
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="C15" s="34" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D15" s="34" t="inlineStr">
+        <is>
+          <t>Find a warm intro before pursuing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>MVPC / other RPCs</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D15" s="35" t="n">
-        <v>40000</v>
-      </c>
-      <c r="E15" s="36" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F15" s="37">
-        <f>IF(AND(ISNUMBER(D15),ISNUMBER(E15)),D15*E15,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="34" t="inlineStr">
-        <is>
-          <t>Qualify</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>MVPC / other RPCs</t>
-        </is>
-      </c>
       <c r="C16" s="34" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>Qualify only once Tier 1 is producing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Community Paradigm (municipal consulting)</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="inlineStr">
+        <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="D16" s="35" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E16" s="36" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F16" s="37">
-        <f>IF(AND(ISNUMBER(D16),ISNUMBER(E16)),D16*E16,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="34" t="inlineStr">
-        <is>
-          <t>Qualify</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Community Paradigm (municipal consulting)</t>
-        </is>
-      </c>
       <c r="C17" s="34" t="inlineStr">
         <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D17" s="35" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E17" s="36" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F17" s="37">
-        <f>IF(AND(ISNUMBER(D17),ISNUMBER(E17)),D17*E17,0)</f>
-        <v/>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>Qualify only once Tier 1 is producing.</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1432,10 +1375,10 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B21:F21"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B25:F25"/>
-    <mergeCell ref="A9:F9"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B22:F22"/>
   </mergeCells>
@@ -1588,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1781,7 +1724,24 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Institutional Stewardship (by itself)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Preventing turnover, lost knowledge, stalled projects, and missed opportunities through Institutional Stewardship</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Always return to the problem. Stewardship disconnected from a real pain point goes abstract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>Tagline, if you need one beneath the wordmark:  Continuity • Data • Stewardship.</t>
         </is>
@@ -1789,7 +1749,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize v1 for launch: consistent price + email, Go-Live checklist, full package
Consistency pass for go-live:
- Permit Path Scan = $500 flat everywhere (docs + site); rush/complex/follow-up
  kept as the run-book ladder.
- Single contact nate@publiclogic.org across site (footer, form, API, start)
  and all docs; ENV_REFERENCE example updated.

New:
- START HERE & Go-Live Checklist doc — package index, what-to-send-whom, the
  go-live steps (domain/email, deploy, wire contact form, E&O gate), and the
  30-day money plan.
- Move Forward "What's in the stack" now lists all current deliverables.

Rebuilt all 14 package docs; workbook formulas validated (0 errors). Web app
typechecks clean and next build prerenders all 15 routes. Public worksheet
download refreshed to the $500 version. Final package = 14 documents.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
+++ b/docs/business/final_deck/PublicLogic - Capabilities Workbook (v2.0 2026-06).xlsx
@@ -2452,7 +2452,7 @@
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>Entry below the Map: the Permit &amp; Bridge tab adds a public-facing ladder — Tier 0 Public Permit Helper (free / very low cost) and Tier 1 Permit Path Scan ($250–$750) — that builds trust and feeds these paid offers.</t>
+          <t>Entry below the Map: the Permit &amp; Bridge tab adds a public-facing ladder — Tier 0 Public Permit Helper (free / very low cost) and Tier 1 Permit Path Scan ($500 flat) — that builds trust and feeds these paid offers.</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>$250 – $750</t>
+          <t>$500 flat</t>
         </is>
       </c>
     </row>

</xml_diff>